<commit_message>
upgrade: update snapshot 20261001;
</commit_message>
<xml_diff>
--- a/snapshot/huobi_por.xlsx
+++ b/snapshot/huobi_por.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2" conformance="strict">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
-  <workbookPr dateCompatibility="0" defaultThemeVersion="202300"/>
+<workbook xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10" conformance="strict">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10414"/>
+  <workbookPr dateCompatibility="0" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Zhuanz/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alef.xu/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C9429CF8-0F2F-9942-957A-803809C69365}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D1568FF8-08EF-2B40-BEB6-0EA6E115364F}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="340" yWindow="500" windowWidth="28100" windowHeight="16560" xr2:uid="{A36C5058-2F1C-3B40-B038-45B73BD959AB}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20620"/>
   </bookViews>
   <sheets>
-    <sheet name="huobi_por" sheetId="1" r:id="rId1"/>
+    <sheet name="huobi_por_副本" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="364" uniqueCount="110">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="387" uniqueCount="113">
   <si>
     <t>coin</t>
   </si>
@@ -72,21 +72,18 @@
     <t>stETH</t>
   </si>
   <si>
+    <t>ETH</t>
+  </si>
+  <si>
     <t>HTX(All)</t>
   </si>
   <si>
-    <t>232059560281012.00</t>
-  </si>
-  <si>
     <t>HTX-ERC20</t>
   </si>
   <si>
     <t>HTX-TRC20</t>
   </si>
   <si>
-    <t>231371738784003.00</t>
-  </si>
-  <si>
     <t>SOL(All)</t>
   </si>
   <si>
@@ -111,7 +108,7 @@
     <t>USDC(All)</t>
   </si>
   <si>
-    <t>USDC-SOL</t>
+    <t>USDC-ERC20</t>
   </si>
   <si>
     <t>U(All)</t>
@@ -129,6 +126,9 @@
     <t>stUSDT-TRC20</t>
   </si>
   <si>
+    <t>jUSDT-TRC20</t>
+  </si>
+  <si>
     <t>USDS(ALL)</t>
   </si>
   <si>
@@ -171,27 +171,21 @@
     <t>IE2P89Qbbay5kzR+mUQyzkJPCF6MpZpt9foZzM63HyKZbe1PegYe7o8qvGA4sIPCQ2VkJuss4vzsMcmyBNK0mRk=</t>
   </si>
   <si>
-    <t>1HckjUpRGcrrRAtFaaCAUaGjsPx9oYmLaZ</t>
+    <t>1LXzGrDQqKqVBqxfGDUyhC6rTRBN5s8Sbj</t>
+  </si>
+  <si>
+    <t>IDxEvxbNOXY2KeARpazYGHu4ZPPx+/LJpG+dItGV1GFNZoR5+sVekMFAf2ICYE0CwULl9PDejDl8aM6fnGheCFM=</t>
+  </si>
+  <si>
+    <t>12AxQ3mM2rwY2mwLa5qNVY65uHoQGfvSVF</t>
+  </si>
+  <si>
+    <t>1AQLXAB6aXSVbRMjbhSBudLf1kcsbWSEjg</t>
   </si>
   <si>
     <t>King will be back!</t>
   </si>
   <si>
-    <t>IJtEWgK2V8QxKUCWpVlfMTpVhwS2My/2Notvcw2lPBuHACHkxUESh8BoPL1vzQ4hkqYg/EZbQm9hpPKKcZJwY7E=</t>
-  </si>
-  <si>
-    <t>1LXzGrDQqKqVBqxfGDUyhC6rTRBN5s8Sbj</t>
-  </si>
-  <si>
-    <t>IDxEvxbNOXY2KeARpazYGHu4ZPPx+/LJpG+dItGV1GFNZoR5+sVekMFAf2ICYE0CwULl9PDejDl8aM6fnGheCFM=</t>
-  </si>
-  <si>
-    <t>12AxQ3mM2rwY2mwLa5qNVY65uHoQGfvSVF</t>
-  </si>
-  <si>
-    <t>1AQLXAB6aXSVbRMjbhSBudLf1kcsbWSEjg</t>
-  </si>
-  <si>
     <t>H1JDQp1uGjVNXcXdpUUUnbiRS1YyttPeo8btOTuA86tXLEIWrVeoNlZsjufIBkfR/f5wqxklyHg1wnNY3cHqIrw=</t>
   </si>
   <si>
@@ -240,7 +234,7 @@
     <t>0x543ae6227abac6fcf74c224d67acab8d84ee2271a839856dd2fba29af42da08d14389f172454d67d60dac16d4cfd72cd6c3c4efc2fa3c5531d4c153e24cb413400</t>
   </si>
   <si>
-    <t>DQhEuTa5UkNcD8YFZK3pvjFfrtMqQpJhSa</t>
+    <t>DLzCvKskasu4Adj3XgbyNitKBukBSa5JPP</t>
   </si>
   <si>
     <t>DRRU8L7fF4k9w7SF3Z6ei8onPCsh9hjGX1</t>
@@ -273,27 +267,39 @@
     <t>DB5KWytcxHyphHPn9iC92Y9JqPRL1Fq21p</t>
   </si>
   <si>
+    <t>DJX3kCZfcDuREturnUNKEBQELi1PFaLkJC</t>
+  </si>
+  <si>
     <t>DP9QNiRnJ1anxwC8LvNPLS1QQc2YoTHd4D</t>
   </si>
   <si>
     <t>D8fLX1YZnMNnDbwi8NbPZ3m3ZUYSHx4DkF</t>
   </si>
   <si>
-    <t>ADwSjbA8Edsk6GHubJnp8vEu9fqHV4PvJ3</t>
+    <t>DK5QPp152bQJxvXmdqiV47H2GZEWApVWUc</t>
+  </si>
+  <si>
+    <t>9zfUDb3bVkVdXUKK9cTDRaKNvTeUX8fyS9</t>
+  </si>
+  <si>
+    <t>DDPRVRRjW1YNupt9mrTekEEEjPHWkVJFiS</t>
   </si>
   <si>
     <t>0x6663613fbd927ce78abbf7f5ca7e2c3fe0d96d18</t>
   </si>
   <si>
+    <t>0x9be5b8a7314552fa47feb1355cd5b4adc7bb7516</t>
+  </si>
+  <si>
+    <t>0xa49abf338f924c7ba547a37a56ad5c22947451fc1171d954ea0793376adfd80d370742f5cdff9e1fd24bf3ba157421854b3e7d80e17d8ad181c56321eadb50641c</t>
+  </si>
+  <si>
     <t>0x18709e89bd403f470088abdacebe86cc60dda12e</t>
   </si>
   <si>
     <t>0x68a79a40adfb16777e49206d60f9cd11de0fbaf3acad5be1e30dd955182475f43255dfec5fede4dc97fcf1fbce1583dd05ee419bf3939ca95919aff931eec41d01</t>
   </si>
   <si>
-    <t>230974428784003.00</t>
-  </si>
-  <si>
     <t>TYh6mgoMNZTCsgpYHBz7gttEfrQmDMABub</t>
   </si>
   <si>
@@ -340,6 +346,9 @@
   </si>
   <si>
     <t>51fbb14497b6f5265b44931dac48e23822b645598d7a9c5fee183c9a517db9491594b82a03e1dfea9072e3e95a29d5716610f5aefdbd934fab8b67d73f148d6900</t>
+  </si>
+  <si>
+    <t>0x9Be5b8A7314552FA47FeB1355CD5b4ADC7Bb7516</t>
   </si>
   <si>
     <t>0xdaa4393013f359fd63a133a3b893d311aba4e471</t>
@@ -360,9 +369,9 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="176" formatCode="0.00_ "/>
+    <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
   </numFmts>
   <fonts count="19">
     <font>
@@ -972,10 +981,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyBorder="1">
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1047,39 +1056,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -1131,7 +1140,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -1242,6 +1251,13 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800%"/>
+        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -1250,13 +1266,6 @@
           <a:miter lim="800%"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800%"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -1321,46 +1330,26 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE4067D0-83EE-2E49-A682-3F955B59A64A}">
-  <dimension ref="A1:F108"/>
+<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F116"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="2" max="2" width="59.1640625" customWidth="1"/>
-    <col min="3" max="3" width="83" customWidth="1"/>
-    <col min="4" max="4" width="34.83203125" customWidth="1"/>
-    <col min="5" max="5" width="13.5" customWidth="1"/>
-    <col min="6" max="6" width="143.33203125" customWidth="1"/>
+    <col min="2" max="2" width="25.6640625" customWidth="1"/>
+    <col min="3" max="3" width="36.6640625" customWidth="1"/>
+    <col min="4" max="4" width="49.33203125" customWidth="1"/>
+    <col min="5" max="5" width="47.33203125" customWidth="1"/>
+    <col min="6" max="6" width="120.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1382,7 +1371,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="1">
-        <v>20252.349999999999</v>
+        <v>20003.96</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1390,10 +1379,10 @@
         <v>5</v>
       </c>
       <c r="B3" s="1">
-        <v>964902</v>
+        <v>969314</v>
       </c>
       <c r="C3" s="1">
-        <v>8083.39</v>
+        <v>7813.99</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1401,10 +1390,10 @@
         <v>6</v>
       </c>
       <c r="B4" s="1">
-        <v>443191405</v>
+        <v>452012013</v>
       </c>
       <c r="C4" s="1">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1412,10 +1401,10 @@
         <v>7</v>
       </c>
       <c r="B5" s="1">
-        <v>85840149</v>
+        <v>86703812</v>
       </c>
       <c r="C5" s="1">
-        <v>10308.93</v>
+        <v>10339.93</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1423,7 +1412,7 @@
         <v>8</v>
       </c>
       <c r="B6" s="1">
-        <v>85840149</v>
+        <v>86703812</v>
       </c>
       <c r="C6" s="1">
         <v>89</v>
@@ -1437,7 +1426,7 @@
         <v>10</v>
       </c>
       <c r="C7" s="1">
-        <v>1689.04</v>
+        <v>1678.04</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1448,7 +1437,7 @@
         <v>4</v>
       </c>
       <c r="C8" s="1">
-        <v>422760583.18000001</v>
+        <v>402197601.5</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1456,10 +1445,10 @@
         <v>12</v>
       </c>
       <c r="B9" s="1">
-        <v>6355057</v>
+        <v>6395942</v>
       </c>
       <c r="C9" s="1">
-        <v>422760583.18000001</v>
+        <v>402197601.5</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1470,7 +1459,7 @@
         <v>4</v>
       </c>
       <c r="C10" s="1">
-        <v>116757.07</v>
+        <v>110550.54</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1478,400 +1467,382 @@
         <v>14</v>
       </c>
       <c r="B11" s="1">
-        <v>25876316</v>
+        <v>26091349</v>
       </c>
       <c r="C11" s="1">
-        <v>29213.08</v>
+        <v>29267.06</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>10</v>
+        <v>15</v>
+      </c>
+      <c r="B12" s="1">
+        <v>26091349</v>
       </c>
       <c r="C12" s="1">
-        <v>87543.99</v>
+        <v>484.25</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="1" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>16</v>
+        <v>10</v>
+      </c>
+      <c r="C13" s="1">
+        <v>80799.23</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B14" s="1">
-        <v>25876316</v>
+        <v>16</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="C14" s="2">
-        <v>386057650000</v>
+        <v>232501767822773</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B15" s="1">
-        <v>85840149</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>19</v>
+        <v>26091349</v>
+      </c>
+      <c r="C15" s="2">
+        <v>386057650000</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>10</v>
+        <v>18</v>
+      </c>
+      <c r="B16" s="1">
+        <v>86703812</v>
       </c>
       <c r="C16" s="2">
-        <v>301763847007.95001</v>
+        <v>231540328784003</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="1" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C17" s="1">
-        <v>401370.12</v>
+        <v>10</v>
+      </c>
+      <c r="C17" s="2">
+        <v>575381388770.14001</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B18" s="1">
-        <v>443191405</v>
+        <v>19</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="C18" s="1">
-        <v>399536.39</v>
+        <v>401176.58</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>10</v>
+        <v>20</v>
+      </c>
+      <c r="B19" s="1">
+        <v>452012013</v>
       </c>
       <c r="C19" s="1">
-        <v>1833.73</v>
+        <v>400994.58</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="1" t="s">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C20" s="1">
-        <v>9384209885.7199993</v>
+        <v>182</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B21" s="1">
-        <v>85840149</v>
+        <v>21</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="C21" s="1">
-        <v>8461736079.7799997</v>
+        <v>9433426237</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B22" s="1">
-        <v>85840149</v>
+        <v>86703812</v>
       </c>
       <c r="C22" s="1">
-        <v>922473805.94000006</v>
+        <v>8510952431</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>4</v>
+        <v>23</v>
+      </c>
+      <c r="B23" s="1">
+        <v>86703812</v>
       </c>
       <c r="C23" s="1">
-        <v>27381853.73</v>
+        <v>922473805.89999998</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B24" s="1">
-        <v>106670116</v>
+        <v>24</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="C24" s="1">
-        <v>27381853.73</v>
+        <v>26171853.73</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>4</v>
+        <v>25</v>
+      </c>
+      <c r="B25" s="1">
+        <v>107340374</v>
       </c>
       <c r="C25" s="1">
-        <v>240401886.12</v>
+        <v>26171853.73</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B26" s="1">
-        <v>443191405</v>
+        <v>26</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="C26" s="1">
-        <v>972000</v>
+        <v>247000810.90000001</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>10</v>
+        <v>27</v>
+      </c>
+      <c r="B27" s="1">
+        <v>26091349</v>
       </c>
       <c r="C27" s="1">
-        <v>239429886.12</v>
+        <v>469632.32</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" s="1" t="s">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C28" s="1">
-        <v>32904965.5</v>
+        <v>246531178.59999999</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B29" s="1">
-        <v>85840149</v>
+        <v>28</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="C29" s="1">
-        <v>14984999</v>
+        <v>37246901.490000002</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>10</v>
+        <v>29</v>
+      </c>
+      <c r="B30" s="1">
+        <v>86703812</v>
       </c>
       <c r="C30" s="1">
-        <v>17919966.5</v>
+        <v>14984999</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" s="1" t="s">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C31" s="1">
-        <v>588327863.60000002</v>
+        <v>22261902.489999998</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B32" s="1">
-        <v>85840149</v>
+        <v>30</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="C32" s="1">
-        <v>1909070.4</v>
+        <v>519591077.10000002</v>
       </c>
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B33" s="1">
-        <v>85840149</v>
+        <v>86703812</v>
       </c>
       <c r="C33" s="1">
-        <v>39548690.640000001</v>
+        <v>1909070.4</v>
       </c>
     </row>
     <row r="34" spans="1:6">
       <c r="A34" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>10</v>
+        <v>32</v>
+      </c>
+      <c r="B34" s="1">
+        <v>86703812</v>
       </c>
       <c r="C34" s="1">
-        <v>546870102.55999994</v>
+        <v>35731194.43</v>
       </c>
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>4</v>
+        <v>33</v>
+      </c>
+      <c r="B35" s="1">
+        <v>86703812</v>
       </c>
       <c r="C35" s="1">
-        <v>360949.9</v>
+        <v>3996048.46</v>
       </c>
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B36" s="1">
-        <v>25876316</v>
+        <v>9</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="C36" s="1">
-        <v>360949.9</v>
+        <v>477954763.80000001</v>
       </c>
     </row>
     <row r="37" spans="1:6">
       <c r="A37" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C37" s="1">
-        <v>131071466.44</v>
+        <v>480000</v>
       </c>
     </row>
     <row r="38" spans="1:6">
       <c r="A38" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B38" s="1">
-        <v>85840149</v>
+        <v>26091349</v>
       </c>
       <c r="C38" s="1">
-        <v>2681000</v>
+        <v>480000</v>
       </c>
     </row>
     <row r="39" spans="1:6">
       <c r="A39" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B39" s="1">
-        <v>85840149</v>
+        <v>36</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="C39" s="1">
-        <v>76466743.670000002</v>
+        <v>134853923.59999999</v>
       </c>
     </row>
     <row r="40" spans="1:6">
       <c r="A40" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B40" s="1">
-        <v>25876316</v>
+        <v>86703812</v>
       </c>
       <c r="C40" s="1">
-        <v>44975772</v>
+        <v>6810336.9000000004</v>
       </c>
     </row>
     <row r="41" spans="1:6">
       <c r="A41" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>10</v>
+        <v>38</v>
+      </c>
+      <c r="B41" s="1">
+        <v>86703812</v>
       </c>
       <c r="C41" s="1">
-        <v>6947950.7699999996</v>
+        <v>76466743.670000002</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="A42" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B42" s="1">
+        <v>26091349</v>
+      </c>
+      <c r="C42" s="1">
+        <v>44975772</v>
       </c>
     </row>
     <row r="43" spans="1:6">
       <c r="A43" s="1" t="s">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E43" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F43" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6">
-      <c r="A44" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C44" s="1">
-        <v>964902</v>
-      </c>
-      <c r="D44" s="1">
-        <v>6132.7</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>45</v>
+        <v>10</v>
+      </c>
+      <c r="C43" s="1">
+        <v>6601071</v>
       </c>
     </row>
     <row r="45" spans="1:6">
       <c r="A45" s="1" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C45" s="1">
-        <v>964902</v>
-      </c>
-      <c r="D45" s="1">
-        <v>970.8</v>
+        <v>40</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>2</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="46" spans="1:6">
@@ -1879,19 +1850,19 @@
         <v>5</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C46" s="1">
-        <v>964902</v>
+        <v>969314</v>
       </c>
       <c r="D46" s="1">
-        <v>8.3800000000000008</v>
+        <v>5862.7</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="47" spans="1:6">
@@ -1899,19 +1870,19 @@
         <v>5</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="C47" s="1">
-        <v>964902</v>
+        <v>969314</v>
       </c>
       <c r="D47" s="1">
-        <v>829.68</v>
+        <v>970.8</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>44</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
     </row>
     <row r="48" spans="1:6">
@@ -1919,19 +1890,19 @@
         <v>5</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="C48" s="1">
-        <v>964902</v>
+        <v>969314</v>
       </c>
       <c r="D48" s="1">
-        <v>80.569999999999993</v>
+        <v>829.68</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>4</v>
+        <v>44</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>4</v>
+        <v>49</v>
       </c>
     </row>
     <row r="49" spans="1:6">
@@ -1939,19 +1910,19 @@
         <v>5</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C49" s="1">
-        <v>964902</v>
+        <v>969314</v>
       </c>
       <c r="D49" s="1">
-        <v>46.26</v>
+        <v>80.569999999999993</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>49</v>
+        <v>4</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>55</v>
+        <v>4</v>
       </c>
     </row>
     <row r="50" spans="1:6">
@@ -1959,33 +1930,33 @@
         <v>5</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="C50" s="1">
-        <v>964902</v>
+        <v>969314</v>
       </c>
       <c r="D50" s="1">
-        <v>15</v>
+        <v>38.25</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>4</v>
+        <v>53</v>
       </c>
     </row>
     <row r="51" spans="1:6">
       <c r="A51" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C51" s="1">
-        <v>443191405</v>
+        <v>969314</v>
       </c>
       <c r="D51" s="1">
-        <v>65</v>
+        <v>32</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>4</v>
@@ -1999,13 +1970,13 @@
         <v>6</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C52" s="1">
-        <v>443191405</v>
+        <v>452012013</v>
       </c>
       <c r="D52" s="1">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>4</v>
@@ -2016,22 +1987,22 @@
     </row>
     <row r="53" spans="1:6">
       <c r="A53" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C53" s="1">
-        <v>85840149</v>
+        <v>452012013</v>
       </c>
       <c r="D53" s="1">
-        <v>10298.93</v>
+        <v>50</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>44</v>
+        <v>4</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>60</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54" spans="1:6">
@@ -2039,19 +2010,19 @@
         <v>7</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C54" s="1">
-        <v>85840149</v>
+        <v>86703812</v>
       </c>
       <c r="D54" s="1">
-        <v>10</v>
+        <v>10298.93</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>4</v>
+        <v>44</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>4</v>
+        <v>58</v>
       </c>
     </row>
     <row r="55" spans="1:6">
@@ -2059,19 +2030,19 @@
         <v>7</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>4</v>
+        <v>59</v>
+      </c>
+      <c r="C55" s="1">
+        <v>86703812</v>
+      </c>
+      <c r="D55" s="1">
+        <v>41</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>63</v>
+        <v>4</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>64</v>
+        <v>4</v>
       </c>
     </row>
     <row r="56" spans="1:6">
@@ -2079,7 +2050,7 @@
         <v>7</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>4</v>
@@ -2088,10 +2059,10 @@
         <v>4</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="57" spans="1:6">
@@ -2099,7 +2070,7 @@
         <v>7</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>4</v>
@@ -2108,10 +2079,10 @@
         <v>4</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="58" spans="1:6">
@@ -2119,7 +2090,7 @@
         <v>7</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>4</v>
@@ -2128,50 +2099,50 @@
         <v>4</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
     </row>
     <row r="59" spans="1:6">
       <c r="A59" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C59" s="1">
-        <v>85840149</v>
-      </c>
-      <c r="D59" s="1">
-        <v>89</v>
+        <v>67</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
     </row>
     <row r="60" spans="1:6">
       <c r="A60" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="C60" s="1">
-        <v>6355057</v>
+        <v>86703812</v>
       </c>
       <c r="D60" s="1">
-        <v>1189758.8700000001</v>
+        <v>89</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>4</v>
+        <v>44</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>4</v>
+        <v>58</v>
       </c>
     </row>
     <row r="61" spans="1:6">
@@ -2179,13 +2150,13 @@
         <v>12</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C61" s="1">
-        <v>6355057</v>
+        <v>6395942</v>
       </c>
       <c r="D61" s="1">
-        <v>342891003.5</v>
+        <v>1089276.1399999999</v>
       </c>
       <c r="E61" s="1" t="s">
         <v>4</v>
@@ -2199,13 +2170,13 @@
         <v>12</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C62" s="1">
-        <v>6355057</v>
+        <v>6395942</v>
       </c>
       <c r="D62" s="1">
-        <v>66066923.390000001</v>
+        <v>310891003.5</v>
       </c>
       <c r="E62" s="1" t="s">
         <v>4</v>
@@ -2219,13 +2190,13 @@
         <v>12</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C63" s="1">
-        <v>6355057</v>
+        <v>6395942</v>
       </c>
       <c r="D63" s="1">
-        <v>2866994</v>
+        <v>66066923.390000001</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>4</v>
@@ -2239,13 +2210,13 @@
         <v>12</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C64" s="1">
-        <v>6355057</v>
+        <v>6395942</v>
       </c>
       <c r="D64" s="1">
-        <v>2647816.5299999998</v>
+        <v>2866994</v>
       </c>
       <c r="E64" s="1" t="s">
         <v>4</v>
@@ -2259,13 +2230,13 @@
         <v>12</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C65" s="1">
-        <v>6355057</v>
+        <v>6395942</v>
       </c>
       <c r="D65" s="1">
-        <v>1457329.63</v>
+        <v>2647816.5299999998</v>
       </c>
       <c r="E65" s="1" t="s">
         <v>4</v>
@@ -2279,13 +2250,13 @@
         <v>12</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C66" s="1">
-        <v>6355057</v>
+        <v>6395942</v>
       </c>
       <c r="D66" s="1">
-        <v>1066964.3</v>
+        <v>1457329.63</v>
       </c>
       <c r="E66" s="1" t="s">
         <v>4</v>
@@ -2299,13 +2270,13 @@
         <v>12</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C67" s="1">
-        <v>6355057</v>
+        <v>6395942</v>
       </c>
       <c r="D67" s="1">
-        <v>850746.71</v>
+        <v>1066964.3</v>
       </c>
       <c r="E67" s="1" t="s">
         <v>4</v>
@@ -2319,13 +2290,13 @@
         <v>12</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C68" s="1">
-        <v>6355057</v>
+        <v>6395942</v>
       </c>
       <c r="D68" s="1">
-        <v>579364.13</v>
+        <v>850746.71</v>
       </c>
       <c r="E68" s="1" t="s">
         <v>4</v>
@@ -2339,13 +2310,13 @@
         <v>12</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C69" s="1">
-        <v>6355057</v>
+        <v>6395942</v>
       </c>
       <c r="D69" s="1">
-        <v>538350.48</v>
+        <v>579364.13</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>4</v>
@@ -2359,13 +2330,13 @@
         <v>12</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C70" s="1">
-        <v>6355057</v>
+        <v>6395942</v>
       </c>
       <c r="D70" s="1">
-        <v>127419.44</v>
+        <v>538350.48</v>
       </c>
       <c r="E70" s="1" t="s">
         <v>4</v>
@@ -2379,13 +2350,13 @@
         <v>12</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C71" s="1">
-        <v>6355057</v>
+        <v>6395942</v>
       </c>
       <c r="D71" s="1">
-        <v>999998.92</v>
+        <v>127419.44</v>
       </c>
       <c r="E71" s="1" t="s">
         <v>4</v>
@@ -2399,13 +2370,13 @@
         <v>12</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C72" s="1">
-        <v>6355057</v>
+        <v>6395942</v>
       </c>
       <c r="D72" s="1">
-        <v>999999.11</v>
+        <v>235415.87</v>
       </c>
       <c r="E72" s="1" t="s">
         <v>4</v>
@@ -2419,13 +2390,13 @@
         <v>12</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C73" s="1">
-        <v>6355057</v>
+        <v>6395942</v>
       </c>
       <c r="D73" s="1">
-        <v>477914.18</v>
+        <v>999998.92</v>
       </c>
       <c r="E73" s="1" t="s">
         <v>4</v>
@@ -2436,16 +2407,16 @@
     </row>
     <row r="74" spans="1:6">
       <c r="A74" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C74" s="1">
-        <v>25876316</v>
+        <v>6395942</v>
       </c>
       <c r="D74" s="1">
-        <v>29213.08</v>
+        <v>999999.11</v>
       </c>
       <c r="E74" s="1" t="s">
         <v>4</v>
@@ -2456,56 +2427,56 @@
     </row>
     <row r="75" spans="1:6">
       <c r="A75" s="1" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C75" s="1">
-        <v>25876316</v>
-      </c>
-      <c r="D75" s="2">
-        <v>386057650000</v>
+        <v>6395942</v>
+      </c>
+      <c r="D75" s="1">
+        <v>999999.38</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>44</v>
+        <v>4</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>87</v>
+        <v>4</v>
       </c>
     </row>
     <row r="76" spans="1:6">
       <c r="A76" s="1" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>59</v>
+        <v>84</v>
       </c>
       <c r="C76" s="1">
-        <v>85840149</v>
-      </c>
-      <c r="D76" s="3" t="s">
-        <v>88</v>
+        <v>6395942</v>
+      </c>
+      <c r="D76" s="1">
+        <v>9780000.4199999999</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>44</v>
+        <v>4</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>60</v>
+        <v>4</v>
       </c>
     </row>
     <row r="77" spans="1:6">
       <c r="A77" s="1" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="C77" s="1">
-        <v>85840149</v>
-      </c>
-      <c r="D77" s="2">
-        <v>397310000000</v>
+        <v>6395942</v>
+      </c>
+      <c r="D77" s="1">
+        <v>999999.52</v>
       </c>
       <c r="E77" s="1" t="s">
         <v>4</v>
@@ -2516,62 +2487,62 @@
     </row>
     <row r="78" spans="1:6">
       <c r="A78" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C78" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D78" s="1" t="s">
-        <v>4</v>
+        <v>86</v>
+      </c>
+      <c r="C78" s="1">
+        <v>26091349</v>
+      </c>
+      <c r="D78" s="1">
+        <v>29267.06</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>63</v>
+        <v>4</v>
       </c>
       <c r="F78" s="1" t="s">
-        <v>64</v>
+        <v>4</v>
       </c>
     </row>
     <row r="79" spans="1:6">
       <c r="A79" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="C79" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D79" s="1" t="s">
-        <v>4</v>
+        <v>87</v>
+      </c>
+      <c r="C79" s="1">
+        <v>26091349</v>
+      </c>
+      <c r="D79" s="1">
+        <v>484.25</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>66</v>
+        <v>88</v>
       </c>
     </row>
     <row r="80" spans="1:6">
       <c r="A80" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="C80" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D80" s="1" t="s">
-        <v>4</v>
+        <v>89</v>
+      </c>
+      <c r="C80" s="1">
+        <v>26091349</v>
+      </c>
+      <c r="D80" s="3">
+        <v>386058000000</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="F80" s="1" t="s">
-        <v>68</v>
+        <v>90</v>
       </c>
     </row>
     <row r="81" spans="1:6">
@@ -2579,33 +2550,33 @@
         <v>18</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="C81" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D81" s="1" t="s">
-        <v>4</v>
+        <v>57</v>
+      </c>
+      <c r="C81" s="1">
+        <v>86703812</v>
+      </c>
+      <c r="D81" s="3">
+        <v>230974000000000</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="F81" s="1" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
     </row>
     <row r="82" spans="1:6">
       <c r="A82" s="1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C82" s="1">
-        <v>443191405</v>
-      </c>
-      <c r="D82" s="1">
-        <v>399536.39</v>
+        <v>86703812</v>
+      </c>
+      <c r="D82" s="3">
+        <v>565900000000</v>
       </c>
       <c r="E82" s="1" t="s">
         <v>4</v>
@@ -2616,296 +2587,296 @@
     </row>
     <row r="83" spans="1:6">
       <c r="A83" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="C83" s="1">
-        <v>85840149</v>
-      </c>
-      <c r="D83" s="1">
-        <v>1082089494.28</v>
+        <v>60</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D83" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F83" s="1" t="s">
-        <v>90</v>
+        <v>62</v>
       </c>
     </row>
     <row r="84" spans="1:6">
       <c r="A84" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="C84" s="1">
-        <v>85840149</v>
-      </c>
-      <c r="D84" s="1">
-        <v>1705110564.0899999</v>
+        <v>63</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F84" s="1" t="s">
-        <v>92</v>
+        <v>64</v>
       </c>
     </row>
     <row r="85" spans="1:6">
       <c r="A85" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C85" s="1">
-        <v>85840149</v>
-      </c>
-      <c r="D85" s="1">
-        <v>755759959.02999997</v>
+        <v>65</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D85" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F85" s="1" t="s">
-        <v>94</v>
+        <v>66</v>
       </c>
     </row>
     <row r="86" spans="1:6">
       <c r="A86" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="C86" s="1">
-        <v>85840149</v>
-      </c>
-      <c r="D86" s="1">
-        <v>1071286648.08</v>
+        <v>67</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D86" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F86" s="1" t="s">
-        <v>96</v>
+        <v>68</v>
       </c>
     </row>
     <row r="87" spans="1:6">
       <c r="A87" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>97</v>
+        <v>55</v>
       </c>
       <c r="C87" s="1">
-        <v>85840149</v>
+        <v>452012013</v>
       </c>
       <c r="D87" s="1">
-        <v>1070397075.17</v>
+        <v>400994.58</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>44</v>
+        <v>4</v>
       </c>
       <c r="F87" s="1" t="s">
-        <v>98</v>
+        <v>4</v>
       </c>
     </row>
     <row r="88" spans="1:6">
       <c r="A88" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C88" s="1">
-        <v>85840149</v>
+        <v>86703812</v>
       </c>
       <c r="D88" s="1">
-        <v>1144452002.4400001</v>
+        <v>1082091198</v>
       </c>
       <c r="E88" s="1" t="s">
         <v>44</v>
       </c>
       <c r="F88" s="1" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
     </row>
     <row r="89" spans="1:6">
       <c r="A89" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>101</v>
+        <v>57</v>
       </c>
       <c r="C89" s="1">
-        <v>85840149</v>
+        <v>86703812</v>
       </c>
       <c r="D89" s="1">
-        <v>1632640336.6900001</v>
+        <v>49207295.030000001</v>
       </c>
       <c r="E89" s="1" t="s">
         <v>44</v>
       </c>
       <c r="F89" s="1" t="s">
-        <v>102</v>
+        <v>58</v>
       </c>
     </row>
     <row r="90" spans="1:6">
       <c r="A90" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="C90" s="1">
-        <v>85840149</v>
+        <v>86703812</v>
       </c>
       <c r="D90" s="1">
-        <v>922473805.94000006</v>
+        <v>1705110564</v>
       </c>
       <c r="E90" s="1" t="s">
         <v>44</v>
       </c>
       <c r="F90" s="1" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
     </row>
     <row r="91" spans="1:6">
       <c r="A91" s="1" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>61</v>
+        <v>95</v>
       </c>
       <c r="C91" s="1">
-        <v>85840149</v>
+        <v>86703812</v>
       </c>
       <c r="D91" s="1">
-        <v>14984999</v>
+        <v>755759959</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>4</v>
+        <v>44</v>
       </c>
       <c r="F91" s="1" t="s">
-        <v>4</v>
+        <v>96</v>
       </c>
     </row>
     <row r="92" spans="1:6">
       <c r="A92" s="1" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C92" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D92" s="1" t="s">
-        <v>4</v>
+        <v>97</v>
+      </c>
+      <c r="C92" s="1">
+        <v>86703812</v>
+      </c>
+      <c r="D92" s="1">
+        <v>1071290324</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="F92" s="1" t="s">
-        <v>64</v>
+        <v>98</v>
       </c>
     </row>
     <row r="93" spans="1:6">
       <c r="A93" s="1" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="C93" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D93" s="1" t="s">
-        <v>4</v>
+        <v>99</v>
+      </c>
+      <c r="C93" s="1">
+        <v>86703812</v>
+      </c>
+      <c r="D93" s="1">
+        <v>1070399047</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="F93" s="1" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
     </row>
     <row r="94" spans="1:6">
       <c r="A94" s="1" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="C94" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D94" s="1" t="s">
-        <v>4</v>
+        <v>101</v>
+      </c>
+      <c r="C94" s="1">
+        <v>86703812</v>
+      </c>
+      <c r="D94" s="1">
+        <v>1144453707</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="F94" s="1" t="s">
-        <v>68</v>
+        <v>102</v>
       </c>
     </row>
     <row r="95" spans="1:6">
       <c r="A95" s="1" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="C95" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D95" s="1" t="s">
-        <v>4</v>
+        <v>103</v>
+      </c>
+      <c r="C95" s="1">
+        <v>86703812</v>
+      </c>
+      <c r="D95" s="1">
+        <v>1632640337</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="F95" s="1" t="s">
-        <v>70</v>
+        <v>104</v>
       </c>
     </row>
     <row r="96" spans="1:6">
       <c r="A96" s="1" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>58</v>
+        <v>105</v>
       </c>
       <c r="C96" s="1">
-        <v>443191405</v>
+        <v>86703812</v>
       </c>
       <c r="D96" s="1">
-        <v>972000</v>
+        <v>922473805.89999998</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>4</v>
+        <v>44</v>
       </c>
       <c r="F96" s="1" t="s">
-        <v>4</v>
+        <v>106</v>
       </c>
     </row>
     <row r="97" spans="1:6">
       <c r="A97" s="1" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C97" s="1">
-        <v>85840149</v>
+        <v>86703812</v>
       </c>
       <c r="D97" s="1">
-        <v>2681000</v>
+        <v>14984999</v>
       </c>
       <c r="E97" s="1" t="s">
         <v>4</v>
@@ -2916,30 +2887,30 @@
     </row>
     <row r="98" spans="1:6">
       <c r="A98" s="1" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="B98" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D98" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E98" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F98" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="C98" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D98" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E98" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="F98" s="1" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="99" spans="1:6">
       <c r="A99" s="1" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C99" s="1" t="s">
         <v>4</v>
@@ -2948,18 +2919,18 @@
         <v>4</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F99" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="100" spans="1:6">
       <c r="A100" s="1" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C100" s="1" t="s">
         <v>4</v>
@@ -2968,18 +2939,18 @@
         <v>4</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F100" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="101" spans="1:6">
       <c r="A101" s="1" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C101" s="1" t="s">
         <v>4</v>
@@ -2988,64 +2959,64 @@
         <v>4</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F101" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="102" spans="1:6">
       <c r="A102" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>59</v>
+        <v>107</v>
       </c>
       <c r="C102" s="1">
-        <v>85840149</v>
+        <v>26091349</v>
       </c>
       <c r="D102" s="1">
-        <v>76466743.670000002</v>
+        <v>469632.32</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="F102" s="1" t="s">
-        <v>60</v>
+        <v>88</v>
       </c>
     </row>
     <row r="103" spans="1:6">
       <c r="A103" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>86</v>
+        <v>57</v>
       </c>
       <c r="C103" s="1">
-        <v>25876316</v>
+        <v>86703812</v>
       </c>
       <c r="D103" s="1">
-        <v>44975772</v>
+        <v>1270336.8999999999</v>
       </c>
       <c r="E103" s="1" t="s">
         <v>44</v>
       </c>
       <c r="F103" s="1" t="s">
-        <v>87</v>
+        <v>58</v>
       </c>
     </row>
     <row r="104" spans="1:6">
       <c r="A104" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>105</v>
+        <v>59</v>
       </c>
       <c r="C104" s="1">
-        <v>25876316</v>
+        <v>86703812</v>
       </c>
       <c r="D104" s="1">
-        <v>360949.9</v>
+        <v>5540000</v>
       </c>
       <c r="E104" s="1" t="s">
         <v>4</v>
@@ -3056,81 +3027,241 @@
     </row>
     <row r="105" spans="1:6">
       <c r="A105" s="1" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C105" s="1">
-        <v>85840149</v>
-      </c>
-      <c r="D105" s="1">
-        <v>1909070.4</v>
+        <v>60</v>
+      </c>
+      <c r="C105" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D105" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F105" s="1" t="s">
-        <v>107</v>
+        <v>62</v>
       </c>
     </row>
     <row r="106" spans="1:6">
       <c r="A106" s="1" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C106" s="1">
-        <v>85840149</v>
-      </c>
-      <c r="D106" s="1">
-        <v>39548690.640000001</v>
+        <v>63</v>
+      </c>
+      <c r="C106" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D106" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="E106" s="1" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F106" s="1" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="107" spans="1:6">
       <c r="A107" s="1" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="C107" s="1">
-        <v>106670116</v>
-      </c>
-      <c r="D107" s="1">
-        <v>26487852.739999998</v>
+        <v>65</v>
+      </c>
+      <c r="C107" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D107" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>4</v>
+        <v>61</v>
       </c>
       <c r="F107" s="1" t="s">
-        <v>4</v>
+        <v>66</v>
       </c>
     </row>
     <row r="108" spans="1:6">
       <c r="A108" s="1" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="B108" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C108" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D108" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E108" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F108" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6">
+      <c r="A109" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C109" s="1">
+        <v>86703812</v>
+      </c>
+      <c r="D109" s="1">
+        <v>76466743.670000002</v>
+      </c>
+      <c r="E109" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F109" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6">
+      <c r="A110" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C110" s="1">
+        <v>26091349</v>
+      </c>
+      <c r="D110" s="1">
+        <v>44975772</v>
+      </c>
+      <c r="E110" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F110" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6">
+      <c r="A111" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C111" s="1">
+        <v>26091349</v>
+      </c>
+      <c r="D111" s="1">
+        <v>480000</v>
+      </c>
+      <c r="E111" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F111" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6">
+      <c r="A112" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B112" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="C108" s="1">
-        <v>106670116</v>
-      </c>
-      <c r="D108" s="1">
-        <v>894000.99</v>
-      </c>
-      <c r="E108" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F108" s="1" t="s">
+      <c r="C112" s="1">
+        <v>86703812</v>
+      </c>
+      <c r="D112" s="1">
+        <v>1909070.4</v>
+      </c>
+      <c r="E112" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F112" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6">
+      <c r="A113" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C113" s="1">
+        <v>86703812</v>
+      </c>
+      <c r="D113" s="1">
+        <v>35731194.43</v>
+      </c>
+      <c r="E113" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F113" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6">
+      <c r="A114" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C114" s="1">
+        <v>86703812</v>
+      </c>
+      <c r="D114" s="1">
+        <v>3996048.46</v>
+      </c>
+      <c r="E114" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F114" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6">
+      <c r="A115" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C115" s="1">
+        <v>107340374</v>
+      </c>
+      <c r="D115" s="1">
+        <v>24987852.739999998</v>
+      </c>
+      <c r="E115" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F115" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6">
+      <c r="A116" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C116" s="1">
+        <v>107340374</v>
+      </c>
+      <c r="D116" s="1">
+        <v>1184000.99</v>
+      </c>
+      <c r="E116" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F116" s="1" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>